<commit_message>
Removed generated files permanently
</commit_message>
<xml_diff>
--- a/TestData/Loans.xlsx
+++ b/TestData/Loans.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="14">
   <si>
     <t>Loan Type</t>
   </si>
@@ -28,37 +28,34 @@
     <t>EMI</t>
   </si>
   <si>
+    <t>Car Loan Advance</t>
+  </si>
+  <si>
+    <t>₹ 1,30,492</t>
+  </si>
+  <si>
+    <t>₹ 0</t>
+  </si>
+  <si>
+    <t>1,30,492</t>
+  </si>
+  <si>
+    <t>Car Loan Arrears</t>
+  </si>
+  <si>
+    <t>₹ 1,19,650</t>
+  </si>
+  <si>
+    <t>₹ 11,875</t>
+  </si>
+  <si>
+    <t>1,31,525</t>
+  </si>
+  <si>
+    <t>Personal Loan</t>
+  </si>
+  <si>
     <t>Home Loan</t>
-  </si>
-  <si>
-    <t>₹ 1,19,650</t>
-  </si>
-  <si>
-    <t>₹ 11,875</t>
-  </si>
-  <si>
-    <t>1,31,525</t>
-  </si>
-  <si>
-    <t>Personal Loan</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Car Loan Advance</t>
-  </si>
-  <si>
-    <t>₹ 1,30,492</t>
-  </si>
-  <si>
-    <t>₹ 0</t>
-  </si>
-  <si>
-    <t>1,30,492</t>
-  </si>
-  <si>
-    <t>Car Loan Arrears</t>
   </si>
 </sst>
 </file>
@@ -122,16 +119,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -160,16 +157,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>9</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -198,30 +195,30 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>